<commit_message>
Update product bulk upload template asset
</commit_message>
<xml_diff>
--- a/src/assets/Tovrika POS Template.xlsx
+++ b/src/assets/Tovrika POS Template.xlsx
@@ -1,21 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{202DE458-0AB6-41EB-AE64-EF0128C11CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="23040" windowHeight="7800"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Products" sheetId="1" r:id="rId1"/>
+    <sheet name="Tags" sheetId="2" r:id="rId2"/>
+    <sheet name="Categories" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -32,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
   <si>
     <t>Product Name</t>
   </si>
@@ -82,6 +79,12 @@
     <t>Is Stock Tracked</t>
   </si>
   <si>
+    <t>Tag Value</t>
+  </si>
+  <si>
+    <t>Category Group Name</t>
+  </si>
+  <si>
     <t>Sample Product</t>
   </si>
   <si>
@@ -97,6 +100,12 @@
     <t>http://example.com/image.jpg</t>
   </si>
   <si>
+    <t>small</t>
+  </si>
+  <si>
+    <t>clothing</t>
+  </si>
+  <si>
     <t>Sample Product 2</t>
   </si>
   <si>
@@ -107,22 +116,218 @@
   </si>
   <si>
     <t>PCODE1234</t>
+  </si>
+  <si>
+    <t>large</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Category Name</t>
+  </si>
+  <si>
+    <t>Beverages</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>This is softdrinks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;₱&quot;* #,##0_-;\-&quot;₱&quot;* #,##0_-;_-&quot;₱&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -141,13 +346,227 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -182,65 +601,323 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFB2B2B2"/>
       </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color rgb="FF000000"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FF7F7F7F"/>
       </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -289,7 +966,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -322,26 +999,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -374,23 +1034,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -532,119 +1175,122 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="14.5740740740741" style="3" customWidth="1"/>
+    <col min="2" max="2" width="18.5740740740741" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.71296296296296" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12.712962962963" style="3" customWidth="1"/>
+    <col min="5" max="5" width="10.4259259259259" style="3" customWidth="1"/>
+    <col min="6" max="6" width="9.42592592592593" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.4259259259259" style="3" customWidth="1"/>
+    <col min="8" max="8" width="11.287037037037" style="3" customWidth="1"/>
+    <col min="9" max="9" width="15" style="4" customWidth="1"/>
+    <col min="10" max="10" width="27.8518518518519" style="3" customWidth="1"/>
+    <col min="11" max="11" width="9.85185185185185" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.8518518518519" style="5" customWidth="1"/>
+    <col min="13" max="13" width="8.85185185185185" style="3" customWidth="1"/>
+    <col min="14" max="14" width="12.1388888888889" style="5" customWidth="1"/>
+    <col min="15" max="15" width="13.8518518518519" style="3" customWidth="1"/>
+    <col min="16" max="16" width="14.8518518518519" style="5" customWidth="1"/>
+    <col min="17" max="17" width="9.55555555555556" style="3" customWidth="1"/>
+    <col min="18" max="18" width="21" style="3" customWidth="1"/>
+    <col min="19" max="16384" width="9.13888888888889" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="7" customFormat="1">
-      <c r="A1" s="4" t="s">
+    <row r="1" s="1" customFormat="1" ht="15.15" spans="1:18">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="7" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:16" s="9" customFormat="1">
-      <c r="A2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="9" t="s">
+    <row r="2" s="2" customFormat="1" spans="1:18">
+      <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="9">
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2">
         <v>100</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="2">
         <v>50</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="2">
         <v>60</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="2">
         <v>70</v>
       </c>
       <c r="I2" s="10">
         <v>1234567890123</v>
       </c>
-      <c r="J2" s="9" t="s">
-        <v>20</v>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="K2" s="11" t="b">
         <v>0</v>
@@ -652,49 +1298,55 @@
       <c r="L2" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M2" s="9">
+      <c r="M2" s="2">
         <v>0</v>
       </c>
       <c r="N2" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="2">
         <v>0</v>
       </c>
       <c r="P2" s="11" t="b">
         <v>1</v>
       </c>
+      <c r="Q2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="3" spans="1:16" ht="30.75">
-      <c r="A3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="9">
+    <row r="3" ht="28.8" spans="1:18">
+      <c r="A3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="2">
         <v>100</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="2">
         <v>50</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="2">
         <v>60</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="2">
         <v>70</v>
       </c>
       <c r="I3" s="10">
         <v>3423424324324</v>
       </c>
-      <c r="J3" s="9" t="s">
-        <v>20</v>
+      <c r="J3" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="K3" s="11" t="b">
         <v>0</v>
@@ -702,34 +1354,126 @@
       <c r="L3" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="2">
         <v>0</v>
       </c>
       <c r="N3" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="2">
         <v>0</v>
       </c>
       <c r="P3" s="11" t="b">
         <v>0</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P1:P1048576 N1:N1048576 K1:L1048576" xr:uid="{9FA0959C-8564-4C40-88B9-92ADB93F2CAC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N$1:N$1048576 P$1:P$1048576 K$1:L$1048576">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12C882B0-9283-4596-B602-75B8E5BB9D3D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="14.8888888888889" customWidth="1"/>
+    <col min="3" max="3" width="15.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix POS store selector deduplication
</commit_message>
<xml_diff>
--- a/src/assets/Tovrika POS Template.xlsx
+++ b/src/assets/Tovrika POS Template.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="7800"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="40">
   <si>
     <t>Product Name</t>
   </si>
@@ -85,10 +85,10 @@
     <t>Category Group Name</t>
   </si>
   <si>
-    <t>Sample Product</t>
-  </si>
-  <si>
-    <t>Sample description</t>
+    <t>Coke</t>
+  </si>
+  <si>
+    <t>Regular Coke</t>
   </si>
   <si>
     <t>SKU123</t>
@@ -103,13 +103,10 @@
     <t>small</t>
   </si>
   <si>
-    <t>clothing</t>
-  </si>
-  <si>
-    <t>Sample Product 2</t>
-  </si>
-  <si>
-    <t>Sample description2</t>
+    <t>Beverages</t>
+  </si>
+  <si>
+    <t>Sprite</t>
   </si>
   <si>
     <t>SKU1234</t>
@@ -146,9 +143,6 @@
   </si>
   <si>
     <t>Category Name</t>
-  </si>
-  <si>
-    <t>Beverages</t>
   </si>
   <si>
     <t>General</t>
@@ -167,14 +161,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -700,148 +687,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1317,18 +1304,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" ht="28.8" spans="1:18">
+    <row r="3" spans="1:18">
       <c r="A3" s="9" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="E3" s="2">
         <v>100</v>
@@ -1367,7 +1354,7 @@
         <v>0</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>24</v>
@@ -1392,46 +1379,46 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
         <v>30</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>34</v>
-      </c>
-      <c r="C2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1452,10 +1439,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1463,13 +1450,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
         <v>39</v>
-      </c>
-      <c r="B2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>